<commit_message>
Part List: Min MAD becomes MAD (optional); new Part Detail sub-menu (TB_M_PART_CROSSDOCK_DTL)
Prototype
- Part List column/field/export/upload: Min MAD -> MAD, optional on Add and Upload
  (filled by the MAD calculation function); Min MAD warning removed
- New Part Detail sub-menu for Procurement (tab next to Part List): CRUD of
  Part Number, Minimum MAD, Case/Day with Add/Edit modal, delete confirmation

UISS
- Part List screen: MAD (TB_M_PART_CANDIDATE.MAD, optional), tab item, new screenshots
- Part List upload: column mad optional (check 5), MAD in data map and table,
  sample scenario N9 (add without MAD)
- Mapping upload: MAD in TB_M_PART_CANDIDATE definition
- New UISS_Screen_PartDetail.xlsx with the TB_M_PART_CROSSDOCK_DTL definition

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/UISS_Batch_PartListUpload_v2.xlsx
+++ b/UISS_Batch_PartListUpload_v2.xlsx
@@ -23970,7 +23970,7 @@
       <c r="S13" s="856" t="n"/>
       <c r="T13" s="1012" t="inlineStr">
         <is>
-          <t>minimum_mad</t>
+          <t>mad</t>
         </is>
       </c>
       <c r="U13" s="855" t="n"/>
@@ -23994,7 +23994,7 @@
       <c r="AN13" s="856" t="n"/>
       <c r="AO13" s="1015" t="inlineStr">
         <is>
-          <t>MIN_MAD</t>
+          <t>MAD</t>
         </is>
       </c>
       <c r="AP13" s="855" t="n"/>
@@ -24007,7 +24007,11 @@
       <c r="AW13" s="855" t="n"/>
       <c r="AX13" s="855" t="n"/>
       <c r="AY13" s="855" t="n"/>
-      <c r="AZ13" s="1015" t="n"/>
+      <c r="AZ13" s="1015" t="inlineStr">
+        <is>
+          <t>Optional; blank = NULL until the MAD calculation function fills it</t>
+        </is>
+      </c>
       <c r="BA13" s="855" t="n"/>
       <c r="BB13" s="855" t="n"/>
       <c r="BC13" s="855" t="n"/>
@@ -28493,7 +28497,7 @@
       <c r="S54" s="856" t="n"/>
       <c r="T54" s="1012" t="inlineStr">
         <is>
-          <t>minimum_mad</t>
+          <t>mad</t>
         </is>
       </c>
       <c r="U54" s="855" t="n"/>
@@ -28517,7 +28521,7 @@
       <c r="AN54" s="856" t="n"/>
       <c r="AO54" s="1015" t="inlineStr">
         <is>
-          <t>MIN_MAD</t>
+          <t>MAD</t>
         </is>
       </c>
       <c r="AP54" s="855" t="n"/>
@@ -28530,7 +28534,11 @@
       <c r="AW54" s="855" t="n"/>
       <c r="AX54" s="855" t="n"/>
       <c r="AY54" s="855" t="n"/>
-      <c r="AZ54" s="1015" t="n"/>
+      <c r="AZ54" s="1015" t="inlineStr">
+        <is>
+          <t>Optional; blank = not changed</t>
+        </is>
+      </c>
       <c r="BA54" s="855" t="n"/>
       <c r="BB54" s="855" t="n"/>
       <c r="BC54" s="855" t="n"/>
@@ -34423,7 +34431,7 @@
       <c r="BD14" s="955" t="n"/>
       <c r="BE14" s="956" t="inlineStr">
         <is>
-          <t>Min MAD (0 or more), Pcs/Case and Max Case/Day (more</t>
+          <t>Pcs/Case and Max Case/Day are whole numbers greater than</t>
         </is>
       </c>
       <c r="BF14" s="957" t="n"/>
@@ -34458,7 +34466,7 @@
       <c r="CI14" s="955" t="n"/>
       <c r="CJ14" s="956" t="inlineStr">
         <is>
-          <t>minimum_mad,</t>
+          <t>pcs_case,</t>
         </is>
       </c>
       <c r="CK14" s="957" t="n"/>
@@ -34536,7 +34544,7 @@
       <c r="BD15" s="959" t="n"/>
       <c r="BE15" s="963" t="inlineStr">
         <is>
-          <t>than 0) are whole numbers. Required on every row, no blank</t>
+          <t>0, required on every row. MAD is optional (filled later by the</t>
         </is>
       </c>
       <c r="BF15" s="961" t="n"/>
@@ -34571,7 +34579,7 @@
       <c r="CI15" s="959" t="n"/>
       <c r="CJ15" s="963" t="inlineStr">
         <is>
-          <t>pcs_case,</t>
+          <t>max_case_day, mad</t>
         </is>
       </c>
       <c r="CK15" s="961" t="n"/>
@@ -34653,7 +34661,7 @@
       <c r="BD16" s="959" t="n"/>
       <c r="BE16" s="963" t="inlineStr">
         <is>
-          <t>cell.</t>
+          <t>MAD calculation function); when filled it is a whole number, 0</t>
         </is>
       </c>
       <c r="BF16" s="961" t="n"/>
@@ -34686,11 +34694,7 @@
       <c r="CG16" s="961" t="n"/>
       <c r="CH16" s="961" t="n"/>
       <c r="CI16" s="959" t="n"/>
-      <c r="CJ16" s="963" t="inlineStr">
-        <is>
-          <t>max_case_day</t>
-        </is>
-      </c>
+      <c r="CJ16" s="963" t="n"/>
       <c r="CK16" s="961" t="n"/>
       <c r="CL16" s="961" t="n"/>
       <c r="CM16" s="961" t="n"/>
@@ -34769,64 +34773,56 @@
       <c r="AY17" s="941" t="n"/>
       <c r="AZ17" s="943" t="n"/>
       <c r="BA17" s="941" t="n"/>
-      <c r="BB17" s="954" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="BC17" s="957" t="n"/>
-      <c r="BD17" s="955" t="n"/>
-      <c r="BE17" s="956" t="inlineStr">
-        <is>
-          <t>Status: flag A must be blank (a new part is always Candidate).</t>
-        </is>
-      </c>
-      <c r="BF17" s="957" t="n"/>
-      <c r="BG17" s="957" t="n"/>
-      <c r="BH17" s="957" t="n"/>
-      <c r="BI17" s="957" t="n"/>
-      <c r="BJ17" s="957" t="n"/>
-      <c r="BK17" s="957" t="n"/>
-      <c r="BL17" s="957" t="n"/>
-      <c r="BM17" s="957" t="n"/>
-      <c r="BN17" s="957" t="n"/>
-      <c r="BO17" s="957" t="n"/>
-      <c r="BP17" s="957" t="n"/>
-      <c r="BQ17" s="957" t="n"/>
-      <c r="BR17" s="957" t="n"/>
-      <c r="BS17" s="957" t="n"/>
-      <c r="BT17" s="957" t="n"/>
-      <c r="BU17" s="957" t="n"/>
-      <c r="BV17" s="957" t="n"/>
-      <c r="BW17" s="957" t="n"/>
-      <c r="BX17" s="957" t="n"/>
-      <c r="BY17" s="957" t="n"/>
-      <c r="BZ17" s="957" t="n"/>
-      <c r="CA17" s="957" t="n"/>
-      <c r="CB17" s="957" t="n"/>
-      <c r="CC17" s="957" t="n"/>
-      <c r="CD17" s="957" t="n"/>
-      <c r="CE17" s="957" t="n"/>
-      <c r="CF17" s="957" t="n"/>
-      <c r="CG17" s="957" t="n"/>
-      <c r="CH17" s="957" t="n"/>
-      <c r="CI17" s="955" t="n"/>
-      <c r="CJ17" s="956" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="CK17" s="957" t="n"/>
-      <c r="CL17" s="957" t="n"/>
-      <c r="CM17" s="957" t="n"/>
-      <c r="CN17" s="957" t="n"/>
-      <c r="CO17" s="957" t="n"/>
-      <c r="CP17" s="957" t="n"/>
-      <c r="CQ17" s="957" t="n"/>
-      <c r="CR17" s="957" t="n"/>
-      <c r="CS17" s="957" t="n"/>
-      <c r="CT17" s="957" t="n"/>
-      <c r="CU17" s="955" t="n"/>
+      <c r="BB17" s="962" t="n"/>
+      <c r="BC17" s="961" t="n"/>
+      <c r="BD17" s="959" t="n"/>
+      <c r="BE17" s="963" t="inlineStr">
+        <is>
+          <t>or more.</t>
+        </is>
+      </c>
+      <c r="BF17" s="961" t="n"/>
+      <c r="BG17" s="961" t="n"/>
+      <c r="BH17" s="961" t="n"/>
+      <c r="BI17" s="961" t="n"/>
+      <c r="BJ17" s="961" t="n"/>
+      <c r="BK17" s="961" t="n"/>
+      <c r="BL17" s="961" t="n"/>
+      <c r="BM17" s="961" t="n"/>
+      <c r="BN17" s="961" t="n"/>
+      <c r="BO17" s="961" t="n"/>
+      <c r="BP17" s="961" t="n"/>
+      <c r="BQ17" s="961" t="n"/>
+      <c r="BR17" s="961" t="n"/>
+      <c r="BS17" s="961" t="n"/>
+      <c r="BT17" s="961" t="n"/>
+      <c r="BU17" s="961" t="n"/>
+      <c r="BV17" s="961" t="n"/>
+      <c r="BW17" s="961" t="n"/>
+      <c r="BX17" s="961" t="n"/>
+      <c r="BY17" s="961" t="n"/>
+      <c r="BZ17" s="961" t="n"/>
+      <c r="CA17" s="961" t="n"/>
+      <c r="CB17" s="961" t="n"/>
+      <c r="CC17" s="961" t="n"/>
+      <c r="CD17" s="961" t="n"/>
+      <c r="CE17" s="961" t="n"/>
+      <c r="CF17" s="961" t="n"/>
+      <c r="CG17" s="961" t="n"/>
+      <c r="CH17" s="961" t="n"/>
+      <c r="CI17" s="959" t="n"/>
+      <c r="CJ17" s="963" t="n"/>
+      <c r="CK17" s="961" t="n"/>
+      <c r="CL17" s="961" t="n"/>
+      <c r="CM17" s="961" t="n"/>
+      <c r="CN17" s="961" t="n"/>
+      <c r="CO17" s="961" t="n"/>
+      <c r="CP17" s="961" t="n"/>
+      <c r="CQ17" s="961" t="n"/>
+      <c r="CR17" s="961" t="n"/>
+      <c r="CS17" s="961" t="n"/>
+      <c r="CT17" s="961" t="n"/>
+      <c r="CU17" s="959" t="n"/>
       <c r="CV17" s="941" t="n"/>
       <c r="CW17" s="941" t="n"/>
       <c r="CX17" s="944" t="n"/>
@@ -34894,56 +34890,64 @@
       <c r="AY18" s="941" t="n"/>
       <c r="AZ18" s="943" t="n"/>
       <c r="BA18" s="941" t="n"/>
-      <c r="BB18" s="962" t="n"/>
-      <c r="BC18" s="961" t="n"/>
-      <c r="BD18" s="959" t="n"/>
-      <c r="BE18" s="963" t="inlineStr">
-        <is>
-          <t>Flag E: a Candidate part must stay Candidate (blank or</t>
-        </is>
-      </c>
-      <c r="BF18" s="961" t="n"/>
-      <c r="BG18" s="961" t="n"/>
-      <c r="BH18" s="961" t="n"/>
-      <c r="BI18" s="961" t="n"/>
-      <c r="BJ18" s="961" t="n"/>
-      <c r="BK18" s="961" t="n"/>
-      <c r="BL18" s="961" t="n"/>
-      <c r="BM18" s="961" t="n"/>
-      <c r="BN18" s="961" t="n"/>
-      <c r="BO18" s="961" t="n"/>
-      <c r="BP18" s="961" t="n"/>
-      <c r="BQ18" s="961" t="n"/>
-      <c r="BR18" s="961" t="n"/>
-      <c r="BS18" s="961" t="n"/>
-      <c r="BT18" s="961" t="n"/>
-      <c r="BU18" s="961" t="n"/>
-      <c r="BV18" s="961" t="n"/>
-      <c r="BW18" s="961" t="n"/>
-      <c r="BX18" s="961" t="n"/>
-      <c r="BY18" s="961" t="n"/>
-      <c r="BZ18" s="961" t="n"/>
-      <c r="CA18" s="961" t="n"/>
-      <c r="CB18" s="961" t="n"/>
-      <c r="CC18" s="961" t="n"/>
-      <c r="CD18" s="961" t="n"/>
-      <c r="CE18" s="961" t="n"/>
-      <c r="CF18" s="961" t="n"/>
-      <c r="CG18" s="961" t="n"/>
-      <c r="CH18" s="961" t="n"/>
-      <c r="CI18" s="959" t="n"/>
-      <c r="CJ18" s="963" t="n"/>
-      <c r="CK18" s="961" t="n"/>
-      <c r="CL18" s="961" t="n"/>
-      <c r="CM18" s="961" t="n"/>
-      <c r="CN18" s="961" t="n"/>
-      <c r="CO18" s="961" t="n"/>
-      <c r="CP18" s="961" t="n"/>
-      <c r="CQ18" s="961" t="n"/>
-      <c r="CR18" s="961" t="n"/>
-      <c r="CS18" s="961" t="n"/>
-      <c r="CT18" s="961" t="n"/>
-      <c r="CU18" s="959" t="n"/>
+      <c r="BB18" s="954" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="BC18" s="957" t="n"/>
+      <c r="BD18" s="955" t="n"/>
+      <c r="BE18" s="956" t="inlineStr">
+        <is>
+          <t>Status: flag A must be blank (a new part is always Candidate).</t>
+        </is>
+      </c>
+      <c r="BF18" s="957" t="n"/>
+      <c r="BG18" s="957" t="n"/>
+      <c r="BH18" s="957" t="n"/>
+      <c r="BI18" s="957" t="n"/>
+      <c r="BJ18" s="957" t="n"/>
+      <c r="BK18" s="957" t="n"/>
+      <c r="BL18" s="957" t="n"/>
+      <c r="BM18" s="957" t="n"/>
+      <c r="BN18" s="957" t="n"/>
+      <c r="BO18" s="957" t="n"/>
+      <c r="BP18" s="957" t="n"/>
+      <c r="BQ18" s="957" t="n"/>
+      <c r="BR18" s="957" t="n"/>
+      <c r="BS18" s="957" t="n"/>
+      <c r="BT18" s="957" t="n"/>
+      <c r="BU18" s="957" t="n"/>
+      <c r="BV18" s="957" t="n"/>
+      <c r="BW18" s="957" t="n"/>
+      <c r="BX18" s="957" t="n"/>
+      <c r="BY18" s="957" t="n"/>
+      <c r="BZ18" s="957" t="n"/>
+      <c r="CA18" s="957" t="n"/>
+      <c r="CB18" s="957" t="n"/>
+      <c r="CC18" s="957" t="n"/>
+      <c r="CD18" s="957" t="n"/>
+      <c r="CE18" s="957" t="n"/>
+      <c r="CF18" s="957" t="n"/>
+      <c r="CG18" s="957" t="n"/>
+      <c r="CH18" s="957" t="n"/>
+      <c r="CI18" s="955" t="n"/>
+      <c r="CJ18" s="956" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="CK18" s="957" t="n"/>
+      <c r="CL18" s="957" t="n"/>
+      <c r="CM18" s="957" t="n"/>
+      <c r="CN18" s="957" t="n"/>
+      <c r="CO18" s="957" t="n"/>
+      <c r="CP18" s="957" t="n"/>
+      <c r="CQ18" s="957" t="n"/>
+      <c r="CR18" s="957" t="n"/>
+      <c r="CS18" s="957" t="n"/>
+      <c r="CT18" s="957" t="n"/>
+      <c r="CU18" s="955" t="n"/>
       <c r="CV18" s="941" t="n"/>
       <c r="CW18" s="941" t="n"/>
       <c r="CX18" s="944" t="n"/>
@@ -35016,7 +35020,7 @@
       <c r="BD19" s="959" t="n"/>
       <c r="BE19" s="963" t="inlineStr">
         <is>
-          <t>Candidate); an Active part may be changed to Inactive and an</t>
+          <t>Flag E: a Candidate part must stay Candidate (blank or</t>
         </is>
       </c>
       <c r="BF19" s="961" t="n"/>
@@ -35133,7 +35137,7 @@
       <c r="BD20" s="959" t="n"/>
       <c r="BE20" s="963" t="inlineStr">
         <is>
-          <t>Inactive part to Active; no part can be changed to Candidate.</t>
+          <t>Candidate); an Active part may be changed to Inactive and an</t>
         </is>
       </c>
       <c r="BF20" s="961" t="n"/>
@@ -35245,64 +35249,56 @@
       <c r="AY21" s="941" t="n"/>
       <c r="AZ21" s="943" t="n"/>
       <c r="BA21" s="941" t="n"/>
-      <c r="BB21" s="954" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="BC21" s="957" t="n"/>
-      <c r="BD21" s="955" t="n"/>
-      <c r="BE21" s="956" t="inlineStr">
-        <is>
-          <t>Effective Start Date is required when the part status is</t>
-        </is>
-      </c>
-      <c r="BF21" s="957" t="n"/>
-      <c r="BG21" s="957" t="n"/>
-      <c r="BH21" s="957" t="n"/>
-      <c r="BI21" s="957" t="n"/>
-      <c r="BJ21" s="957" t="n"/>
-      <c r="BK21" s="957" t="n"/>
-      <c r="BL21" s="957" t="n"/>
-      <c r="BM21" s="957" t="n"/>
-      <c r="BN21" s="957" t="n"/>
-      <c r="BO21" s="957" t="n"/>
-      <c r="BP21" s="957" t="n"/>
-      <c r="BQ21" s="957" t="n"/>
-      <c r="BR21" s="957" t="n"/>
-      <c r="BS21" s="957" t="n"/>
-      <c r="BT21" s="957" t="n"/>
-      <c r="BU21" s="957" t="n"/>
-      <c r="BV21" s="957" t="n"/>
-      <c r="BW21" s="957" t="n"/>
-      <c r="BX21" s="957" t="n"/>
-      <c r="BY21" s="957" t="n"/>
-      <c r="BZ21" s="957" t="n"/>
-      <c r="CA21" s="957" t="n"/>
-      <c r="CB21" s="957" t="n"/>
-      <c r="CC21" s="957" t="n"/>
-      <c r="CD21" s="957" t="n"/>
-      <c r="CE21" s="957" t="n"/>
-      <c r="CF21" s="957" t="n"/>
-      <c r="CG21" s="957" t="n"/>
-      <c r="CH21" s="957" t="n"/>
-      <c r="CI21" s="955" t="n"/>
-      <c r="CJ21" s="956" t="inlineStr">
-        <is>
-          <t>effective_start_date</t>
-        </is>
-      </c>
-      <c r="CK21" s="957" t="n"/>
-      <c r="CL21" s="957" t="n"/>
-      <c r="CM21" s="957" t="n"/>
-      <c r="CN21" s="957" t="n"/>
-      <c r="CO21" s="957" t="n"/>
-      <c r="CP21" s="957" t="n"/>
-      <c r="CQ21" s="957" t="n"/>
-      <c r="CR21" s="957" t="n"/>
-      <c r="CS21" s="957" t="n"/>
-      <c r="CT21" s="957" t="n"/>
-      <c r="CU21" s="955" t="n"/>
+      <c r="BB21" s="962" t="n"/>
+      <c r="BC21" s="961" t="n"/>
+      <c r="BD21" s="959" t="n"/>
+      <c r="BE21" s="963" t="inlineStr">
+        <is>
+          <t>Inactive part to Active; no part can be changed to Candidate.</t>
+        </is>
+      </c>
+      <c r="BF21" s="961" t="n"/>
+      <c r="BG21" s="961" t="n"/>
+      <c r="BH21" s="961" t="n"/>
+      <c r="BI21" s="961" t="n"/>
+      <c r="BJ21" s="961" t="n"/>
+      <c r="BK21" s="961" t="n"/>
+      <c r="BL21" s="961" t="n"/>
+      <c r="BM21" s="961" t="n"/>
+      <c r="BN21" s="961" t="n"/>
+      <c r="BO21" s="961" t="n"/>
+      <c r="BP21" s="961" t="n"/>
+      <c r="BQ21" s="961" t="n"/>
+      <c r="BR21" s="961" t="n"/>
+      <c r="BS21" s="961" t="n"/>
+      <c r="BT21" s="961" t="n"/>
+      <c r="BU21" s="961" t="n"/>
+      <c r="BV21" s="961" t="n"/>
+      <c r="BW21" s="961" t="n"/>
+      <c r="BX21" s="961" t="n"/>
+      <c r="BY21" s="961" t="n"/>
+      <c r="BZ21" s="961" t="n"/>
+      <c r="CA21" s="961" t="n"/>
+      <c r="CB21" s="961" t="n"/>
+      <c r="CC21" s="961" t="n"/>
+      <c r="CD21" s="961" t="n"/>
+      <c r="CE21" s="961" t="n"/>
+      <c r="CF21" s="961" t="n"/>
+      <c r="CG21" s="961" t="n"/>
+      <c r="CH21" s="961" t="n"/>
+      <c r="CI21" s="959" t="n"/>
+      <c r="CJ21" s="963" t="n"/>
+      <c r="CK21" s="961" t="n"/>
+      <c r="CL21" s="961" t="n"/>
+      <c r="CM21" s="961" t="n"/>
+      <c r="CN21" s="961" t="n"/>
+      <c r="CO21" s="961" t="n"/>
+      <c r="CP21" s="961" t="n"/>
+      <c r="CQ21" s="961" t="n"/>
+      <c r="CR21" s="961" t="n"/>
+      <c r="CS21" s="961" t="n"/>
+      <c r="CT21" s="961" t="n"/>
+      <c r="CU21" s="959" t="n"/>
       <c r="CV21" s="941" t="n"/>
       <c r="CW21" s="941" t="n"/>
       <c r="CX21" s="944" t="n"/>
@@ -35362,56 +35358,64 @@
       <c r="AY22" s="941" t="n"/>
       <c r="AZ22" s="943" t="n"/>
       <c r="BA22" s="941" t="n"/>
-      <c r="BB22" s="962" t="n"/>
-      <c r="BC22" s="961" t="n"/>
-      <c r="BD22" s="959" t="n"/>
-      <c r="BE22" s="963" t="inlineStr">
-        <is>
-          <t>Candidate (always for flag A) and must be today or later when</t>
-        </is>
-      </c>
-      <c r="BF22" s="961" t="n"/>
-      <c r="BG22" s="961" t="n"/>
-      <c r="BH22" s="961" t="n"/>
-      <c r="BI22" s="961" t="n"/>
-      <c r="BJ22" s="961" t="n"/>
-      <c r="BK22" s="961" t="n"/>
-      <c r="BL22" s="961" t="n"/>
-      <c r="BM22" s="961" t="n"/>
-      <c r="BN22" s="961" t="n"/>
-      <c r="BO22" s="961" t="n"/>
-      <c r="BP22" s="961" t="n"/>
-      <c r="BQ22" s="961" t="n"/>
-      <c r="BR22" s="961" t="n"/>
-      <c r="BS22" s="961" t="n"/>
-      <c r="BT22" s="961" t="n"/>
-      <c r="BU22" s="961" t="n"/>
-      <c r="BV22" s="961" t="n"/>
-      <c r="BW22" s="961" t="n"/>
-      <c r="BX22" s="961" t="n"/>
-      <c r="BY22" s="961" t="n"/>
-      <c r="BZ22" s="961" t="n"/>
-      <c r="CA22" s="961" t="n"/>
-      <c r="CB22" s="961" t="n"/>
-      <c r="CC22" s="961" t="n"/>
-      <c r="CD22" s="961" t="n"/>
-      <c r="CE22" s="961" t="n"/>
-      <c r="CF22" s="961" t="n"/>
-      <c r="CG22" s="961" t="n"/>
-      <c r="CH22" s="961" t="n"/>
-      <c r="CI22" s="959" t="n"/>
-      <c r="CJ22" s="963" t="n"/>
-      <c r="CK22" s="961" t="n"/>
-      <c r="CL22" s="961" t="n"/>
-      <c r="CM22" s="961" t="n"/>
-      <c r="CN22" s="961" t="n"/>
-      <c r="CO22" s="961" t="n"/>
-      <c r="CP22" s="961" t="n"/>
-      <c r="CQ22" s="961" t="n"/>
-      <c r="CR22" s="961" t="n"/>
-      <c r="CS22" s="961" t="n"/>
-      <c r="CT22" s="961" t="n"/>
-      <c r="CU22" s="959" t="n"/>
+      <c r="BB22" s="954" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="BC22" s="957" t="n"/>
+      <c r="BD22" s="955" t="n"/>
+      <c r="BE22" s="956" t="inlineStr">
+        <is>
+          <t>Effective Start Date is required when the part status is</t>
+        </is>
+      </c>
+      <c r="BF22" s="957" t="n"/>
+      <c r="BG22" s="957" t="n"/>
+      <c r="BH22" s="957" t="n"/>
+      <c r="BI22" s="957" t="n"/>
+      <c r="BJ22" s="957" t="n"/>
+      <c r="BK22" s="957" t="n"/>
+      <c r="BL22" s="957" t="n"/>
+      <c r="BM22" s="957" t="n"/>
+      <c r="BN22" s="957" t="n"/>
+      <c r="BO22" s="957" t="n"/>
+      <c r="BP22" s="957" t="n"/>
+      <c r="BQ22" s="957" t="n"/>
+      <c r="BR22" s="957" t="n"/>
+      <c r="BS22" s="957" t="n"/>
+      <c r="BT22" s="957" t="n"/>
+      <c r="BU22" s="957" t="n"/>
+      <c r="BV22" s="957" t="n"/>
+      <c r="BW22" s="957" t="n"/>
+      <c r="BX22" s="957" t="n"/>
+      <c r="BY22" s="957" t="n"/>
+      <c r="BZ22" s="957" t="n"/>
+      <c r="CA22" s="957" t="n"/>
+      <c r="CB22" s="957" t="n"/>
+      <c r="CC22" s="957" t="n"/>
+      <c r="CD22" s="957" t="n"/>
+      <c r="CE22" s="957" t="n"/>
+      <c r="CF22" s="957" t="n"/>
+      <c r="CG22" s="957" t="n"/>
+      <c r="CH22" s="957" t="n"/>
+      <c r="CI22" s="955" t="n"/>
+      <c r="CJ22" s="956" t="inlineStr">
+        <is>
+          <t>effective_start_date</t>
+        </is>
+      </c>
+      <c r="CK22" s="957" t="n"/>
+      <c r="CL22" s="957" t="n"/>
+      <c r="CM22" s="957" t="n"/>
+      <c r="CN22" s="957" t="n"/>
+      <c r="CO22" s="957" t="n"/>
+      <c r="CP22" s="957" t="n"/>
+      <c r="CQ22" s="957" t="n"/>
+      <c r="CR22" s="957" t="n"/>
+      <c r="CS22" s="957" t="n"/>
+      <c r="CT22" s="957" t="n"/>
+      <c r="CU22" s="955" t="n"/>
       <c r="CV22" s="941" t="n"/>
       <c r="CW22" s="941" t="n"/>
       <c r="CX22" s="944" t="n"/>
@@ -35480,7 +35484,7 @@
       <c r="BD23" s="959" t="n"/>
       <c r="BE23" s="963" t="inlineStr">
         <is>
-          <t>new or changed.</t>
+          <t>Candidate (always for flag A) and must be today or later when</t>
         </is>
       </c>
       <c r="BF23" s="961" t="n"/>
@@ -35588,64 +35592,56 @@
       <c r="AY24" s="941" t="n"/>
       <c r="AZ24" s="943" t="n"/>
       <c r="BA24" s="941" t="n"/>
-      <c r="BB24" s="954" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="BC24" s="957" t="n"/>
-      <c r="BD24" s="955" t="n"/>
-      <c r="BE24" s="956" t="inlineStr">
-        <is>
-          <t>Flag E: Effective Start Date can only change while the part</t>
-        </is>
-      </c>
-      <c r="BF24" s="957" t="n"/>
-      <c r="BG24" s="957" t="n"/>
-      <c r="BH24" s="957" t="n"/>
-      <c r="BI24" s="957" t="n"/>
-      <c r="BJ24" s="957" t="n"/>
-      <c r="BK24" s="957" t="n"/>
-      <c r="BL24" s="957" t="n"/>
-      <c r="BM24" s="957" t="n"/>
-      <c r="BN24" s="957" t="n"/>
-      <c r="BO24" s="957" t="n"/>
-      <c r="BP24" s="957" t="n"/>
-      <c r="BQ24" s="957" t="n"/>
-      <c r="BR24" s="957" t="n"/>
-      <c r="BS24" s="957" t="n"/>
-      <c r="BT24" s="957" t="n"/>
-      <c r="BU24" s="957" t="n"/>
-      <c r="BV24" s="957" t="n"/>
-      <c r="BW24" s="957" t="n"/>
-      <c r="BX24" s="957" t="n"/>
-      <c r="BY24" s="957" t="n"/>
-      <c r="BZ24" s="957" t="n"/>
-      <c r="CA24" s="957" t="n"/>
-      <c r="CB24" s="957" t="n"/>
-      <c r="CC24" s="957" t="n"/>
-      <c r="CD24" s="957" t="n"/>
-      <c r="CE24" s="957" t="n"/>
-      <c r="CF24" s="957" t="n"/>
-      <c r="CG24" s="957" t="n"/>
-      <c r="CH24" s="957" t="n"/>
-      <c r="CI24" s="955" t="n"/>
-      <c r="CJ24" s="956" t="inlineStr">
-        <is>
-          <t>effective_start_date</t>
-        </is>
-      </c>
-      <c r="CK24" s="957" t="n"/>
-      <c r="CL24" s="957" t="n"/>
-      <c r="CM24" s="957" t="n"/>
-      <c r="CN24" s="957" t="n"/>
-      <c r="CO24" s="957" t="n"/>
-      <c r="CP24" s="957" t="n"/>
-      <c r="CQ24" s="957" t="n"/>
-      <c r="CR24" s="957" t="n"/>
-      <c r="CS24" s="957" t="n"/>
-      <c r="CT24" s="957" t="n"/>
-      <c r="CU24" s="955" t="n"/>
+      <c r="BB24" s="962" t="n"/>
+      <c r="BC24" s="961" t="n"/>
+      <c r="BD24" s="959" t="n"/>
+      <c r="BE24" s="963" t="inlineStr">
+        <is>
+          <t>new or changed.</t>
+        </is>
+      </c>
+      <c r="BF24" s="961" t="n"/>
+      <c r="BG24" s="961" t="n"/>
+      <c r="BH24" s="961" t="n"/>
+      <c r="BI24" s="961" t="n"/>
+      <c r="BJ24" s="961" t="n"/>
+      <c r="BK24" s="961" t="n"/>
+      <c r="BL24" s="961" t="n"/>
+      <c r="BM24" s="961" t="n"/>
+      <c r="BN24" s="961" t="n"/>
+      <c r="BO24" s="961" t="n"/>
+      <c r="BP24" s="961" t="n"/>
+      <c r="BQ24" s="961" t="n"/>
+      <c r="BR24" s="961" t="n"/>
+      <c r="BS24" s="961" t="n"/>
+      <c r="BT24" s="961" t="n"/>
+      <c r="BU24" s="961" t="n"/>
+      <c r="BV24" s="961" t="n"/>
+      <c r="BW24" s="961" t="n"/>
+      <c r="BX24" s="961" t="n"/>
+      <c r="BY24" s="961" t="n"/>
+      <c r="BZ24" s="961" t="n"/>
+      <c r="CA24" s="961" t="n"/>
+      <c r="CB24" s="961" t="n"/>
+      <c r="CC24" s="961" t="n"/>
+      <c r="CD24" s="961" t="n"/>
+      <c r="CE24" s="961" t="n"/>
+      <c r="CF24" s="961" t="n"/>
+      <c r="CG24" s="961" t="n"/>
+      <c r="CH24" s="961" t="n"/>
+      <c r="CI24" s="959" t="n"/>
+      <c r="CJ24" s="963" t="n"/>
+      <c r="CK24" s="961" t="n"/>
+      <c r="CL24" s="961" t="n"/>
+      <c r="CM24" s="961" t="n"/>
+      <c r="CN24" s="961" t="n"/>
+      <c r="CO24" s="961" t="n"/>
+      <c r="CP24" s="961" t="n"/>
+      <c r="CQ24" s="961" t="n"/>
+      <c r="CR24" s="961" t="n"/>
+      <c r="CS24" s="961" t="n"/>
+      <c r="CT24" s="961" t="n"/>
+      <c r="CU24" s="959" t="n"/>
       <c r="CV24" s="941" t="n"/>
       <c r="CW24" s="941" t="n"/>
       <c r="CX24" s="944" t="n"/>
@@ -35705,56 +35701,64 @@
       <c r="AY25" s="941" t="n"/>
       <c r="AZ25" s="943" t="n"/>
       <c r="BA25" s="941" t="n"/>
-      <c r="BB25" s="962" t="n"/>
-      <c r="BC25" s="961" t="n"/>
-      <c r="BD25" s="959" t="n"/>
-      <c r="BE25" s="963" t="inlineStr">
-        <is>
-          <t>status is Candidate.</t>
-        </is>
-      </c>
-      <c r="BF25" s="961" t="n"/>
-      <c r="BG25" s="961" t="n"/>
-      <c r="BH25" s="961" t="n"/>
-      <c r="BI25" s="961" t="n"/>
-      <c r="BJ25" s="961" t="n"/>
-      <c r="BK25" s="961" t="n"/>
-      <c r="BL25" s="961" t="n"/>
-      <c r="BM25" s="961" t="n"/>
-      <c r="BN25" s="961" t="n"/>
-      <c r="BO25" s="961" t="n"/>
-      <c r="BP25" s="961" t="n"/>
-      <c r="BQ25" s="961" t="n"/>
-      <c r="BR25" s="961" t="n"/>
-      <c r="BS25" s="961" t="n"/>
-      <c r="BT25" s="961" t="n"/>
-      <c r="BU25" s="961" t="n"/>
-      <c r="BV25" s="961" t="n"/>
-      <c r="BW25" s="961" t="n"/>
-      <c r="BX25" s="961" t="n"/>
-      <c r="BY25" s="961" t="n"/>
-      <c r="BZ25" s="961" t="n"/>
-      <c r="CA25" s="961" t="n"/>
-      <c r="CB25" s="961" t="n"/>
-      <c r="CC25" s="961" t="n"/>
-      <c r="CD25" s="961" t="n"/>
-      <c r="CE25" s="961" t="n"/>
-      <c r="CF25" s="961" t="n"/>
-      <c r="CG25" s="961" t="n"/>
-      <c r="CH25" s="961" t="n"/>
-      <c r="CI25" s="959" t="n"/>
-      <c r="CJ25" s="963" t="n"/>
-      <c r="CK25" s="961" t="n"/>
-      <c r="CL25" s="961" t="n"/>
-      <c r="CM25" s="961" t="n"/>
-      <c r="CN25" s="961" t="n"/>
-      <c r="CO25" s="961" t="n"/>
-      <c r="CP25" s="961" t="n"/>
-      <c r="CQ25" s="961" t="n"/>
-      <c r="CR25" s="961" t="n"/>
-      <c r="CS25" s="961" t="n"/>
-      <c r="CT25" s="961" t="n"/>
-      <c r="CU25" s="959" t="n"/>
+      <c r="BB25" s="954" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="BC25" s="957" t="n"/>
+      <c r="BD25" s="955" t="n"/>
+      <c r="BE25" s="956" t="inlineStr">
+        <is>
+          <t>Flag E: Effective Start Date can only change while the part</t>
+        </is>
+      </c>
+      <c r="BF25" s="957" t="n"/>
+      <c r="BG25" s="957" t="n"/>
+      <c r="BH25" s="957" t="n"/>
+      <c r="BI25" s="957" t="n"/>
+      <c r="BJ25" s="957" t="n"/>
+      <c r="BK25" s="957" t="n"/>
+      <c r="BL25" s="957" t="n"/>
+      <c r="BM25" s="957" t="n"/>
+      <c r="BN25" s="957" t="n"/>
+      <c r="BO25" s="957" t="n"/>
+      <c r="BP25" s="957" t="n"/>
+      <c r="BQ25" s="957" t="n"/>
+      <c r="BR25" s="957" t="n"/>
+      <c r="BS25" s="957" t="n"/>
+      <c r="BT25" s="957" t="n"/>
+      <c r="BU25" s="957" t="n"/>
+      <c r="BV25" s="957" t="n"/>
+      <c r="BW25" s="957" t="n"/>
+      <c r="BX25" s="957" t="n"/>
+      <c r="BY25" s="957" t="n"/>
+      <c r="BZ25" s="957" t="n"/>
+      <c r="CA25" s="957" t="n"/>
+      <c r="CB25" s="957" t="n"/>
+      <c r="CC25" s="957" t="n"/>
+      <c r="CD25" s="957" t="n"/>
+      <c r="CE25" s="957" t="n"/>
+      <c r="CF25" s="957" t="n"/>
+      <c r="CG25" s="957" t="n"/>
+      <c r="CH25" s="957" t="n"/>
+      <c r="CI25" s="955" t="n"/>
+      <c r="CJ25" s="956" t="inlineStr">
+        <is>
+          <t>effective_start_date</t>
+        </is>
+      </c>
+      <c r="CK25" s="957" t="n"/>
+      <c r="CL25" s="957" t="n"/>
+      <c r="CM25" s="957" t="n"/>
+      <c r="CN25" s="957" t="n"/>
+      <c r="CO25" s="957" t="n"/>
+      <c r="CP25" s="957" t="n"/>
+      <c r="CQ25" s="957" t="n"/>
+      <c r="CR25" s="957" t="n"/>
+      <c r="CS25" s="957" t="n"/>
+      <c r="CT25" s="957" t="n"/>
+      <c r="CU25" s="955" t="n"/>
       <c r="CV25" s="941" t="n"/>
       <c r="CW25" s="941" t="n"/>
       <c r="CX25" s="944" t="n"/>
@@ -35818,64 +35822,56 @@
       <c r="AY26" s="941" t="n"/>
       <c r="AZ26" s="943" t="n"/>
       <c r="BA26" s="941" t="n"/>
-      <c r="BB26" s="954" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="BC26" s="957" t="n"/>
-      <c r="BD26" s="955" t="n"/>
-      <c r="BE26" s="956" t="inlineStr">
-        <is>
-          <t>Flag E: Max Case/Day is not below the total Case/Day already</t>
-        </is>
-      </c>
-      <c r="BF26" s="957" t="n"/>
-      <c r="BG26" s="957" t="n"/>
-      <c r="BH26" s="957" t="n"/>
-      <c r="BI26" s="957" t="n"/>
-      <c r="BJ26" s="957" t="n"/>
-      <c r="BK26" s="957" t="n"/>
-      <c r="BL26" s="957" t="n"/>
-      <c r="BM26" s="957" t="n"/>
-      <c r="BN26" s="957" t="n"/>
-      <c r="BO26" s="957" t="n"/>
-      <c r="BP26" s="957" t="n"/>
-      <c r="BQ26" s="957" t="n"/>
-      <c r="BR26" s="957" t="n"/>
-      <c r="BS26" s="957" t="n"/>
-      <c r="BT26" s="957" t="n"/>
-      <c r="BU26" s="957" t="n"/>
-      <c r="BV26" s="957" t="n"/>
-      <c r="BW26" s="957" t="n"/>
-      <c r="BX26" s="957" t="n"/>
-      <c r="BY26" s="957" t="n"/>
-      <c r="BZ26" s="957" t="n"/>
-      <c r="CA26" s="957" t="n"/>
-      <c r="CB26" s="957" t="n"/>
-      <c r="CC26" s="957" t="n"/>
-      <c r="CD26" s="957" t="n"/>
-      <c r="CE26" s="957" t="n"/>
-      <c r="CF26" s="957" t="n"/>
-      <c r="CG26" s="957" t="n"/>
-      <c r="CH26" s="957" t="n"/>
-      <c r="CI26" s="955" t="n"/>
-      <c r="CJ26" s="956" t="inlineStr">
-        <is>
-          <t>max_case_day</t>
-        </is>
-      </c>
-      <c r="CK26" s="957" t="n"/>
-      <c r="CL26" s="957" t="n"/>
-      <c r="CM26" s="957" t="n"/>
-      <c r="CN26" s="957" t="n"/>
-      <c r="CO26" s="957" t="n"/>
-      <c r="CP26" s="957" t="n"/>
-      <c r="CQ26" s="957" t="n"/>
-      <c r="CR26" s="957" t="n"/>
-      <c r="CS26" s="957" t="n"/>
-      <c r="CT26" s="957" t="n"/>
-      <c r="CU26" s="955" t="n"/>
+      <c r="BB26" s="962" t="n"/>
+      <c r="BC26" s="961" t="n"/>
+      <c r="BD26" s="959" t="n"/>
+      <c r="BE26" s="963" t="inlineStr">
+        <is>
+          <t>status is Candidate.</t>
+        </is>
+      </c>
+      <c r="BF26" s="961" t="n"/>
+      <c r="BG26" s="961" t="n"/>
+      <c r="BH26" s="961" t="n"/>
+      <c r="BI26" s="961" t="n"/>
+      <c r="BJ26" s="961" t="n"/>
+      <c r="BK26" s="961" t="n"/>
+      <c r="BL26" s="961" t="n"/>
+      <c r="BM26" s="961" t="n"/>
+      <c r="BN26" s="961" t="n"/>
+      <c r="BO26" s="961" t="n"/>
+      <c r="BP26" s="961" t="n"/>
+      <c r="BQ26" s="961" t="n"/>
+      <c r="BR26" s="961" t="n"/>
+      <c r="BS26" s="961" t="n"/>
+      <c r="BT26" s="961" t="n"/>
+      <c r="BU26" s="961" t="n"/>
+      <c r="BV26" s="961" t="n"/>
+      <c r="BW26" s="961" t="n"/>
+      <c r="BX26" s="961" t="n"/>
+      <c r="BY26" s="961" t="n"/>
+      <c r="BZ26" s="961" t="n"/>
+      <c r="CA26" s="961" t="n"/>
+      <c r="CB26" s="961" t="n"/>
+      <c r="CC26" s="961" t="n"/>
+      <c r="CD26" s="961" t="n"/>
+      <c r="CE26" s="961" t="n"/>
+      <c r="CF26" s="961" t="n"/>
+      <c r="CG26" s="961" t="n"/>
+      <c r="CH26" s="961" t="n"/>
+      <c r="CI26" s="959" t="n"/>
+      <c r="CJ26" s="963" t="n"/>
+      <c r="CK26" s="961" t="n"/>
+      <c r="CL26" s="961" t="n"/>
+      <c r="CM26" s="961" t="n"/>
+      <c r="CN26" s="961" t="n"/>
+      <c r="CO26" s="961" t="n"/>
+      <c r="CP26" s="961" t="n"/>
+      <c r="CQ26" s="961" t="n"/>
+      <c r="CR26" s="961" t="n"/>
+      <c r="CS26" s="961" t="n"/>
+      <c r="CT26" s="961" t="n"/>
+      <c r="CU26" s="959" t="n"/>
       <c r="CV26" s="941" t="n"/>
       <c r="CW26" s="941" t="n"/>
       <c r="CX26" s="944" t="n"/>
@@ -35943,56 +35939,64 @@
       <c r="AY27" s="941" t="n"/>
       <c r="AZ27" s="943" t="n"/>
       <c r="BA27" s="941" t="n"/>
-      <c r="BB27" s="962" t="n"/>
-      <c r="BC27" s="961" t="n"/>
-      <c r="BD27" s="959" t="n"/>
-      <c r="BE27" s="963" t="inlineStr">
-        <is>
-          <t>mapped per destination in the ongoing calculation period of</t>
-        </is>
-      </c>
-      <c r="BF27" s="961" t="n"/>
-      <c r="BG27" s="961" t="n"/>
-      <c r="BH27" s="961" t="n"/>
-      <c r="BI27" s="961" t="n"/>
-      <c r="BJ27" s="961" t="n"/>
-      <c r="BK27" s="961" t="n"/>
-      <c r="BL27" s="961" t="n"/>
-      <c r="BM27" s="961" t="n"/>
-      <c r="BN27" s="961" t="n"/>
-      <c r="BO27" s="961" t="n"/>
-      <c r="BP27" s="961" t="n"/>
-      <c r="BQ27" s="961" t="n"/>
-      <c r="BR27" s="961" t="n"/>
-      <c r="BS27" s="961" t="n"/>
-      <c r="BT27" s="961" t="n"/>
-      <c r="BU27" s="961" t="n"/>
-      <c r="BV27" s="961" t="n"/>
-      <c r="BW27" s="961" t="n"/>
-      <c r="BX27" s="961" t="n"/>
-      <c r="BY27" s="961" t="n"/>
-      <c r="BZ27" s="961" t="n"/>
-      <c r="CA27" s="961" t="n"/>
-      <c r="CB27" s="961" t="n"/>
-      <c r="CC27" s="961" t="n"/>
-      <c r="CD27" s="961" t="n"/>
-      <c r="CE27" s="961" t="n"/>
-      <c r="CF27" s="961" t="n"/>
-      <c r="CG27" s="961" t="n"/>
-      <c r="CH27" s="961" t="n"/>
-      <c r="CI27" s="959" t="n"/>
-      <c r="CJ27" s="963" t="n"/>
-      <c r="CK27" s="961" t="n"/>
-      <c r="CL27" s="961" t="n"/>
-      <c r="CM27" s="961" t="n"/>
-      <c r="CN27" s="961" t="n"/>
-      <c r="CO27" s="961" t="n"/>
-      <c r="CP27" s="961" t="n"/>
-      <c r="CQ27" s="961" t="n"/>
-      <c r="CR27" s="961" t="n"/>
-      <c r="CS27" s="961" t="n"/>
-      <c r="CT27" s="961" t="n"/>
-      <c r="CU27" s="959" t="n"/>
+      <c r="BB27" s="954" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="BC27" s="957" t="n"/>
+      <c r="BD27" s="955" t="n"/>
+      <c r="BE27" s="956" t="inlineStr">
+        <is>
+          <t>Flag E: Max Case/Day is not below the total Case/Day already</t>
+        </is>
+      </c>
+      <c r="BF27" s="957" t="n"/>
+      <c r="BG27" s="957" t="n"/>
+      <c r="BH27" s="957" t="n"/>
+      <c r="BI27" s="957" t="n"/>
+      <c r="BJ27" s="957" t="n"/>
+      <c r="BK27" s="957" t="n"/>
+      <c r="BL27" s="957" t="n"/>
+      <c r="BM27" s="957" t="n"/>
+      <c r="BN27" s="957" t="n"/>
+      <c r="BO27" s="957" t="n"/>
+      <c r="BP27" s="957" t="n"/>
+      <c r="BQ27" s="957" t="n"/>
+      <c r="BR27" s="957" t="n"/>
+      <c r="BS27" s="957" t="n"/>
+      <c r="BT27" s="957" t="n"/>
+      <c r="BU27" s="957" t="n"/>
+      <c r="BV27" s="957" t="n"/>
+      <c r="BW27" s="957" t="n"/>
+      <c r="BX27" s="957" t="n"/>
+      <c r="BY27" s="957" t="n"/>
+      <c r="BZ27" s="957" t="n"/>
+      <c r="CA27" s="957" t="n"/>
+      <c r="CB27" s="957" t="n"/>
+      <c r="CC27" s="957" t="n"/>
+      <c r="CD27" s="957" t="n"/>
+      <c r="CE27" s="957" t="n"/>
+      <c r="CF27" s="957" t="n"/>
+      <c r="CG27" s="957" t="n"/>
+      <c r="CH27" s="957" t="n"/>
+      <c r="CI27" s="955" t="n"/>
+      <c r="CJ27" s="956" t="inlineStr">
+        <is>
+          <t>max_case_day</t>
+        </is>
+      </c>
+      <c r="CK27" s="957" t="n"/>
+      <c r="CL27" s="957" t="n"/>
+      <c r="CM27" s="957" t="n"/>
+      <c r="CN27" s="957" t="n"/>
+      <c r="CO27" s="957" t="n"/>
+      <c r="CP27" s="957" t="n"/>
+      <c r="CQ27" s="957" t="n"/>
+      <c r="CR27" s="957" t="n"/>
+      <c r="CS27" s="957" t="n"/>
+      <c r="CT27" s="957" t="n"/>
+      <c r="CU27" s="955" t="n"/>
       <c r="CV27" s="941" t="n"/>
       <c r="CW27" s="941" t="n"/>
       <c r="CX27" s="944" t="n"/>
@@ -36061,7 +36065,7 @@
       <c r="BD28" s="959" t="n"/>
       <c r="BE28" s="963" t="inlineStr">
         <is>
-          <t>Mapping per Destination (TB_M_PART_CANDIDATE_DEST)</t>
+          <t>mapped per destination in the ongoing calculation period of</t>
         </is>
       </c>
       <c r="BF28" s="961" t="n"/>
@@ -36178,7 +36182,7 @@
       <c r="BD29" s="959" t="n"/>
       <c r="BE29" s="963" t="inlineStr">
         <is>
-          <t>(e.g. mapped 100, new Max Case/Day 80 is rejected). The</t>
+          <t>Mapping per Destination (TB_M_PART_CANDIDATE_DEST)</t>
         </is>
       </c>
       <c r="BF29" s="961" t="n"/>
@@ -36291,7 +36295,7 @@
       <c r="BD30" s="959" t="n"/>
       <c r="BE30" s="963" t="inlineStr">
         <is>
-          <t>user must first reduce the mapping in the Mapping per</t>
+          <t>(e.g. mapped 100, new Max Case/Day 80 is rejected). The</t>
         </is>
       </c>
       <c r="BF30" s="961" t="n"/>
@@ -36399,56 +36403,56 @@
       <c r="AY31" s="941" t="n"/>
       <c r="AZ31" s="943" t="n"/>
       <c r="BA31" s="941" t="n"/>
-      <c r="BB31" s="969" t="n"/>
-      <c r="BC31" s="972" t="n"/>
-      <c r="BD31" s="970" t="n"/>
-      <c r="BE31" s="975" t="inlineStr">
-        <is>
-          <t>Destination sub-menu, then lower Max Case/Day in Part List.</t>
-        </is>
-      </c>
-      <c r="BF31" s="972" t="n"/>
-      <c r="BG31" s="972" t="n"/>
-      <c r="BH31" s="972" t="n"/>
-      <c r="BI31" s="972" t="n"/>
-      <c r="BJ31" s="972" t="n"/>
-      <c r="BK31" s="972" t="n"/>
-      <c r="BL31" s="972" t="n"/>
-      <c r="BM31" s="972" t="n"/>
-      <c r="BN31" s="972" t="n"/>
-      <c r="BO31" s="972" t="n"/>
-      <c r="BP31" s="972" t="n"/>
-      <c r="BQ31" s="972" t="n"/>
-      <c r="BR31" s="972" t="n"/>
-      <c r="BS31" s="972" t="n"/>
-      <c r="BT31" s="972" t="n"/>
-      <c r="BU31" s="972" t="n"/>
-      <c r="BV31" s="972" t="n"/>
-      <c r="BW31" s="972" t="n"/>
-      <c r="BX31" s="972" t="n"/>
-      <c r="BY31" s="972" t="n"/>
-      <c r="BZ31" s="972" t="n"/>
-      <c r="CA31" s="972" t="n"/>
-      <c r="CB31" s="972" t="n"/>
-      <c r="CC31" s="972" t="n"/>
-      <c r="CD31" s="972" t="n"/>
-      <c r="CE31" s="972" t="n"/>
-      <c r="CF31" s="972" t="n"/>
-      <c r="CG31" s="972" t="n"/>
-      <c r="CH31" s="972" t="n"/>
-      <c r="CI31" s="970" t="n"/>
-      <c r="CJ31" s="975" t="n"/>
-      <c r="CK31" s="972" t="n"/>
-      <c r="CL31" s="972" t="n"/>
-      <c r="CM31" s="972" t="n"/>
-      <c r="CN31" s="972" t="n"/>
-      <c r="CO31" s="972" t="n"/>
-      <c r="CP31" s="972" t="n"/>
-      <c r="CQ31" s="972" t="n"/>
-      <c r="CR31" s="972" t="n"/>
-      <c r="CS31" s="972" t="n"/>
-      <c r="CT31" s="972" t="n"/>
-      <c r="CU31" s="970" t="n"/>
+      <c r="BB31" s="962" t="n"/>
+      <c r="BC31" s="961" t="n"/>
+      <c r="BD31" s="959" t="n"/>
+      <c r="BE31" s="963" t="inlineStr">
+        <is>
+          <t>user must first reduce the mapping in the Mapping per</t>
+        </is>
+      </c>
+      <c r="BF31" s="961" t="n"/>
+      <c r="BG31" s="961" t="n"/>
+      <c r="BH31" s="961" t="n"/>
+      <c r="BI31" s="961" t="n"/>
+      <c r="BJ31" s="961" t="n"/>
+      <c r="BK31" s="961" t="n"/>
+      <c r="BL31" s="961" t="n"/>
+      <c r="BM31" s="961" t="n"/>
+      <c r="BN31" s="961" t="n"/>
+      <c r="BO31" s="961" t="n"/>
+      <c r="BP31" s="961" t="n"/>
+      <c r="BQ31" s="961" t="n"/>
+      <c r="BR31" s="961" t="n"/>
+      <c r="BS31" s="961" t="n"/>
+      <c r="BT31" s="961" t="n"/>
+      <c r="BU31" s="961" t="n"/>
+      <c r="BV31" s="961" t="n"/>
+      <c r="BW31" s="961" t="n"/>
+      <c r="BX31" s="961" t="n"/>
+      <c r="BY31" s="961" t="n"/>
+      <c r="BZ31" s="961" t="n"/>
+      <c r="CA31" s="961" t="n"/>
+      <c r="CB31" s="961" t="n"/>
+      <c r="CC31" s="961" t="n"/>
+      <c r="CD31" s="961" t="n"/>
+      <c r="CE31" s="961" t="n"/>
+      <c r="CF31" s="961" t="n"/>
+      <c r="CG31" s="961" t="n"/>
+      <c r="CH31" s="961" t="n"/>
+      <c r="CI31" s="959" t="n"/>
+      <c r="CJ31" s="963" t="n"/>
+      <c r="CK31" s="961" t="n"/>
+      <c r="CL31" s="961" t="n"/>
+      <c r="CM31" s="961" t="n"/>
+      <c r="CN31" s="961" t="n"/>
+      <c r="CO31" s="961" t="n"/>
+      <c r="CP31" s="961" t="n"/>
+      <c r="CQ31" s="961" t="n"/>
+      <c r="CR31" s="961" t="n"/>
+      <c r="CS31" s="961" t="n"/>
+      <c r="CT31" s="961" t="n"/>
+      <c r="CU31" s="959" t="n"/>
       <c r="CV31" s="941" t="n"/>
       <c r="CW31" s="941" t="n"/>
       <c r="CX31" s="944" t="n"/>
@@ -36516,52 +36520,56 @@
       <c r="AY32" s="941" t="n"/>
       <c r="AZ32" s="943" t="n"/>
       <c r="BA32" s="941" t="n"/>
-      <c r="BB32" s="941" t="n"/>
-      <c r="BC32" s="941" t="n"/>
-      <c r="BD32" s="941" t="n"/>
-      <c r="BE32" s="941" t="n"/>
-      <c r="BF32" s="941" t="n"/>
-      <c r="BG32" s="941" t="n"/>
-      <c r="BH32" s="941" t="n"/>
-      <c r="BI32" s="941" t="n"/>
-      <c r="BJ32" s="941" t="n"/>
-      <c r="BK32" s="941" t="n"/>
-      <c r="BL32" s="941" t="n"/>
-      <c r="BM32" s="941" t="n"/>
-      <c r="BN32" s="941" t="n"/>
-      <c r="BO32" s="941" t="n"/>
-      <c r="BP32" s="941" t="n"/>
-      <c r="BQ32" s="941" t="n"/>
-      <c r="BR32" s="941" t="n"/>
-      <c r="BS32" s="941" t="n"/>
-      <c r="BT32" s="941" t="n"/>
-      <c r="BU32" s="941" t="n"/>
-      <c r="BV32" s="941" t="n"/>
-      <c r="BW32" s="941" t="n"/>
-      <c r="BX32" s="941" t="n"/>
-      <c r="BY32" s="941" t="n"/>
-      <c r="BZ32" s="941" t="n"/>
-      <c r="CA32" s="941" t="n"/>
-      <c r="CB32" s="941" t="n"/>
-      <c r="CC32" s="941" t="n"/>
-      <c r="CD32" s="941" t="n"/>
-      <c r="CE32" s="941" t="n"/>
-      <c r="CF32" s="941" t="n"/>
-      <c r="CG32" s="941" t="n"/>
-      <c r="CH32" s="941" t="n"/>
-      <c r="CI32" s="941" t="n"/>
-      <c r="CJ32" s="941" t="n"/>
-      <c r="CK32" s="941" t="n"/>
-      <c r="CL32" s="941" t="n"/>
-      <c r="CM32" s="941" t="n"/>
-      <c r="CN32" s="941" t="n"/>
-      <c r="CO32" s="941" t="n"/>
-      <c r="CP32" s="941" t="n"/>
-      <c r="CQ32" s="941" t="n"/>
-      <c r="CR32" s="941" t="n"/>
-      <c r="CS32" s="941" t="n"/>
-      <c r="CT32" s="941" t="n"/>
-      <c r="CU32" s="941" t="n"/>
+      <c r="BB32" s="969" t="n"/>
+      <c r="BC32" s="972" t="n"/>
+      <c r="BD32" s="970" t="n"/>
+      <c r="BE32" s="975" t="inlineStr">
+        <is>
+          <t>Destination sub-menu, then lower Max Case/Day in Part List.</t>
+        </is>
+      </c>
+      <c r="BF32" s="972" t="n"/>
+      <c r="BG32" s="972" t="n"/>
+      <c r="BH32" s="972" t="n"/>
+      <c r="BI32" s="972" t="n"/>
+      <c r="BJ32" s="972" t="n"/>
+      <c r="BK32" s="972" t="n"/>
+      <c r="BL32" s="972" t="n"/>
+      <c r="BM32" s="972" t="n"/>
+      <c r="BN32" s="972" t="n"/>
+      <c r="BO32" s="972" t="n"/>
+      <c r="BP32" s="972" t="n"/>
+      <c r="BQ32" s="972" t="n"/>
+      <c r="BR32" s="972" t="n"/>
+      <c r="BS32" s="972" t="n"/>
+      <c r="BT32" s="972" t="n"/>
+      <c r="BU32" s="972" t="n"/>
+      <c r="BV32" s="972" t="n"/>
+      <c r="BW32" s="972" t="n"/>
+      <c r="BX32" s="972" t="n"/>
+      <c r="BY32" s="972" t="n"/>
+      <c r="BZ32" s="972" t="n"/>
+      <c r="CA32" s="972" t="n"/>
+      <c r="CB32" s="972" t="n"/>
+      <c r="CC32" s="972" t="n"/>
+      <c r="CD32" s="972" t="n"/>
+      <c r="CE32" s="972" t="n"/>
+      <c r="CF32" s="972" t="n"/>
+      <c r="CG32" s="972" t="n"/>
+      <c r="CH32" s="972" t="n"/>
+      <c r="CI32" s="970" t="n"/>
+      <c r="CJ32" s="975" t="n"/>
+      <c r="CK32" s="972" t="n"/>
+      <c r="CL32" s="972" t="n"/>
+      <c r="CM32" s="972" t="n"/>
+      <c r="CN32" s="972" t="n"/>
+      <c r="CO32" s="972" t="n"/>
+      <c r="CP32" s="972" t="n"/>
+      <c r="CQ32" s="972" t="n"/>
+      <c r="CR32" s="972" t="n"/>
+      <c r="CS32" s="972" t="n"/>
+      <c r="CT32" s="972" t="n"/>
+      <c r="CU32" s="970" t="n"/>
       <c r="CV32" s="941" t="n"/>
       <c r="CW32" s="941" t="n"/>
       <c r="CX32" s="944" t="n"/>
@@ -38272,7 +38280,7 @@
       <c r="CY48" s="941" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="95">
+  <mergeCells count="98">
     <mergeCell ref="CJ8:CU8"/>
     <mergeCell ref="BE12:CI12"/>
     <mergeCell ref="CJ26:CU26"/>
@@ -38315,6 +38323,7 @@
     <mergeCell ref="BE29:CI29"/>
     <mergeCell ref="BB28:BD28"/>
     <mergeCell ref="CC3:CJ3"/>
+    <mergeCell ref="BE32:CI32"/>
     <mergeCell ref="BB30:BD30"/>
     <mergeCell ref="BB15:BD15"/>
     <mergeCell ref="BB29:BD29"/>
@@ -38359,6 +38368,8 @@
     <mergeCell ref="BB21:BD21"/>
     <mergeCell ref="BE18:CI18"/>
     <mergeCell ref="CC4:CJ4"/>
+    <mergeCell ref="BB32:BD32"/>
+    <mergeCell ref="CJ32:CU32"/>
     <mergeCell ref="BB13:BD13"/>
     <mergeCell ref="CJ13:CU13"/>
     <mergeCell ref="BB16:BD16"/>
@@ -44492,7 +44503,7 @@
       <c r="B11" s="942" t="n"/>
       <c r="C11" s="956" t="inlineStr">
         <is>
-          <t>minimum_mad</t>
+          <t>mad</t>
         </is>
       </c>
       <c r="D11" s="957" t="n"/>
@@ -44512,7 +44523,7 @@
       <c r="R11" s="955" t="n"/>
       <c r="S11" s="956" t="inlineStr">
         <is>
-          <t>Minimum MAD</t>
+          <t>MAD (optional; filled later by the MAD calculation function)</t>
         </is>
       </c>
       <c r="T11" s="957" t="n"/>
@@ -46298,7 +46309,7 @@
       <c r="D27" s="941" t="n"/>
       <c r="E27" s="966" t="inlineStr">
         <is>
-          <t>MIN_MAD</t>
+          <t>MAD</t>
         </is>
       </c>
       <c r="F27" s="957" t="n"/>
@@ -46337,7 +46348,7 @@
       <c r="AI27" s="955" t="n"/>
       <c r="AJ27" s="965" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="AK27" s="957" t="n"/>
@@ -46345,7 +46356,7 @@
       <c r="AM27" s="955" t="n"/>
       <c r="AN27" s="956" t="inlineStr">
         <is>
-          <t>Minimum MAD</t>
+          <t>MAD; result of the MAD calculation function, optional on Add / Upload</t>
         </is>
       </c>
       <c r="AO27" s="957" t="n"/>
@@ -48987,7 +48998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="710" min="1" max="1"/>
@@ -49043,7 +49054,7 @@
       </c>
       <c r="C6" s="1052" t="inlineStr">
         <is>
-          <t>Min MAD</t>
+          <t>MAD</t>
         </is>
       </c>
       <c r="D6" s="1052" t="inlineStr">
@@ -49305,7 +49316,7 @@
       </c>
       <c r="D16" s="1052" t="inlineStr">
         <is>
-          <t>minimum_mad</t>
+          <t>mad</t>
         </is>
       </c>
       <c r="E16" s="1052" t="inlineStr">
@@ -49675,268 +49686,262 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1051" t="inlineStr">
-        <is>
-          <t>C. Error scenarios (whole file rejected, nothing saved)</t>
+    <row r="25">
+      <c r="A25" s="1053" t="inlineStr">
+        <is>
+          <t>N9</t>
+        </is>
+      </c>
+      <c r="B25" s="1053" t="inlineStr">
+        <is>
+          <t>Add a new part without MAD</t>
+        </is>
+      </c>
+      <c r="C25" s="1053" t="inlineStr">
+        <is>
+          <t>PART-M03</t>
+        </is>
+      </c>
+      <c r="D25" s="1053" t="n"/>
+      <c r="E25" s="1054" t="n">
+        <v>25</v>
+      </c>
+      <c r="F25" s="1054" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="1053" t="n"/>
+      <c r="H25" s="1053" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I25" s="1053" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="J25" s="1053" t="inlineStr">
+        <is>
+          <t>Inserted. MAD stays blank until the MAD calculation function fills it.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1052" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B27" s="1052" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C27" s="1052" t="inlineStr">
-        <is>
-          <t>part_no</t>
-        </is>
-      </c>
-      <c r="D27" s="1052" t="inlineStr">
-        <is>
-          <t>minimum_mad</t>
-        </is>
-      </c>
-      <c r="E27" s="1052" t="inlineStr">
-        <is>
-          <t>pcs_case</t>
-        </is>
-      </c>
-      <c r="F27" s="1052" t="inlineStr">
-        <is>
-          <t>max_case_day</t>
-        </is>
-      </c>
-      <c r="G27" s="1052" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="H27" s="1052" t="inlineStr">
-        <is>
-          <t>flag_add_edit</t>
-        </is>
-      </c>
-      <c r="I27" s="1052" t="inlineStr">
-        <is>
-          <t>effective_start_date</t>
-        </is>
-      </c>
-      <c r="J27" s="1052" t="inlineStr">
-        <is>
-          <t>Error (4.2 check no.)</t>
+      <c r="A27" s="1051" t="inlineStr">
+        <is>
+          <t>C. Error scenarios (whole file rejected, nothing saved)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1053" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B28" s="1053" t="inlineStr">
-        <is>
-          <t>Flag is not A or E</t>
-        </is>
-      </c>
-      <c r="C28" s="1053" t="inlineStr">
-        <is>
-          <t>PART-I</t>
-        </is>
-      </c>
-      <c r="D28" s="1054" t="n">
-        <v>300</v>
-      </c>
-      <c r="E28" s="1054" t="n">
-        <v>15</v>
-      </c>
-      <c r="F28" s="1054" t="n">
-        <v>18</v>
-      </c>
-      <c r="G28" s="1053" t="n"/>
-      <c r="H28" s="1053" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I28" s="1053" t="inlineStr">
-        <is>
-          <t>20-Sep-2026</t>
-        </is>
-      </c>
-      <c r="J28" s="1053" t="inlineStr">
-        <is>
-          <t>Check 1: flag_add_edit must be A or E.</t>
+      <c r="A28" s="1052" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B28" s="1052" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C28" s="1052" t="inlineStr">
+        <is>
+          <t>part_no</t>
+        </is>
+      </c>
+      <c r="D28" s="1052" t="inlineStr">
+        <is>
+          <t>mad</t>
+        </is>
+      </c>
+      <c r="E28" s="1052" t="inlineStr">
+        <is>
+          <t>pcs_case</t>
+        </is>
+      </c>
+      <c r="F28" s="1052" t="inlineStr">
+        <is>
+          <t>max_case_day</t>
+        </is>
+      </c>
+      <c r="G28" s="1052" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H28" s="1052" t="inlineStr">
+        <is>
+          <t>flag_add_edit</t>
+        </is>
+      </c>
+      <c r="I28" s="1052" t="inlineStr">
+        <is>
+          <t>effective_start_date</t>
+        </is>
+      </c>
+      <c r="J28" s="1052" t="inlineStr">
+        <is>
+          <t>Error (4.2 check no.)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1053" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B29" s="1053" t="inlineStr">
         <is>
-          <t>Part not in part master</t>
+          <t>Flag is not A or E</t>
         </is>
       </c>
       <c r="C29" s="1053" t="inlineStr">
         <is>
-          <t>PART-Z99</t>
+          <t>PART-I</t>
         </is>
       </c>
       <c r="D29" s="1054" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E29" s="1054" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F29" s="1054" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G29" s="1053" t="n"/>
       <c r="H29" s="1053" t="inlineStr">
         <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="I29" s="1053" t="n"/>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I29" s="1053" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="J29" s="1053" t="inlineStr">
         <is>
-          <t>Check 2: Part No not found in TB_M_PART_MASTER.</t>
+          <t>Check 1: flag_add_edit must be A or E.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1053" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B30" s="1053" t="inlineStr">
         <is>
-          <t>Add a part that is already registered</t>
+          <t>Part not in part master</t>
         </is>
       </c>
       <c r="C30" s="1053" t="inlineStr">
         <is>
-          <t>PART-A</t>
+          <t>PART-Z99</t>
         </is>
       </c>
       <c r="D30" s="1054" t="n">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="E30" s="1054" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F30" s="1054" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G30" s="1053" t="n"/>
       <c r="H30" s="1053" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I30" s="1053" t="inlineStr">
-        <is>
-          <t>14-Sep-2026</t>
-        </is>
-      </c>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="I30" s="1053" t="n"/>
       <c r="J30" s="1053" t="inlineStr">
         <is>
-          <t>Check 3: Part No already registered, use flag E.</t>
+          <t>Check 2: Part No not found in TB_M_PART_MASTER.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1053" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B31" s="1053" t="inlineStr">
         <is>
-          <t>Edit a part that is not registered</t>
+          <t>Add a part that is already registered</t>
         </is>
       </c>
       <c r="C31" s="1053" t="inlineStr">
         <is>
-          <t>PART-M03</t>
+          <t>PART-A</t>
         </is>
       </c>
       <c r="D31" s="1054" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="E31" s="1054" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F31" s="1054" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="G31" s="1053" t="n"/>
       <c r="H31" s="1053" t="inlineStr">
         <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="I31" s="1053" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I31" s="1053" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
       <c r="J31" s="1053" t="inlineStr">
         <is>
-          <t>Check 3: Part No not registered, use flag A.</t>
+          <t>Check 3: Part No already registered, use flag E.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1053" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B32" s="1053" t="inlineStr">
         <is>
-          <t>Same part twice in the file (row 1)</t>
+          <t>Edit a part that is not registered</t>
         </is>
       </c>
       <c r="C32" s="1053" t="inlineStr">
         <is>
-          <t>PART-I</t>
+          <t>PART-M03</t>
         </is>
       </c>
       <c r="D32" s="1054" t="n">
         <v>300</v>
       </c>
       <c r="E32" s="1054" t="n">
+        <v>20</v>
+      </c>
+      <c r="F32" s="1054" t="n">
         <v>15</v>
       </c>
-      <c r="F32" s="1054" t="n">
-        <v>18</v>
-      </c>
-      <c r="G32" s="1053" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
+      <c r="G32" s="1053" t="n"/>
       <c r="H32" s="1053" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="I32" s="1053" t="inlineStr">
-        <is>
-          <t>20-Sep-2026</t>
-        </is>
-      </c>
+      <c r="I32" s="1053" t="n"/>
       <c r="J32" s="1053" t="inlineStr">
         <is>
-          <t>Check 4: Part No appears more than once.</t>
+          <t>Check 3: Part No not registered, use flag A.</t>
         </is>
       </c>
     </row>
@@ -49948,7 +49953,7 @@
       </c>
       <c r="B33" s="1053" t="inlineStr">
         <is>
-          <t>Same part twice in the file (row 2)</t>
+          <t>Same part twice in the file (row 1)</t>
         </is>
       </c>
       <c r="C33" s="1053" t="inlineStr">
@@ -49963,7 +49968,7 @@
         <v>15</v>
       </c>
       <c r="F33" s="1054" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G33" s="1053" t="inlineStr">
         <is>
@@ -49989,119 +49994,119 @@
     <row r="34">
       <c r="A34" s="1053" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B34" s="1053" t="inlineStr">
         <is>
-          <t>Invalid number</t>
+          <t>Same part twice in the file (row 2)</t>
         </is>
       </c>
       <c r="C34" s="1053" t="inlineStr">
         <is>
-          <t>PART-M03</t>
+          <t>PART-I</t>
         </is>
       </c>
       <c r="D34" s="1054" t="n">
         <v>300</v>
       </c>
       <c r="E34" s="1054" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F34" s="1054" t="n">
-        <v>15</v>
-      </c>
-      <c r="G34" s="1053" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="G34" s="1053" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
       <c r="H34" s="1053" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I34" s="1053" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="J34" s="1053" t="inlineStr">
         <is>
-          <t>Check 5: pcs_case must be greater than 0. A blank cell in a required column is also an error.</t>
+          <t>Check 4: Part No appears more than once.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1053" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B35" s="1053" t="inlineStr">
         <is>
-          <t>Change the status of a Candidate part</t>
+          <t>Invalid number</t>
         </is>
       </c>
       <c r="C35" s="1053" t="inlineStr">
         <is>
-          <t>PART-I</t>
+          <t>PART-M03</t>
         </is>
       </c>
       <c r="D35" s="1054" t="n">
         <v>300</v>
       </c>
       <c r="E35" s="1054" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1054" t="n">
         <v>15</v>
       </c>
-      <c r="F35" s="1054" t="n">
-        <v>20</v>
-      </c>
-      <c r="G35" s="1053" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="G35" s="1053" t="n"/>
       <c r="H35" s="1053" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I35" s="1053" t="inlineStr">
         <is>
-          <t>15-Sep-2026</t>
+          <t>14-Sep-2026</t>
         </is>
       </c>
       <c r="J35" s="1053" t="inlineStr">
         <is>
-          <t>Check 6: the status of a Candidate part cannot be changed by upload. Change it in the Edit part data modal.</t>
+          <t>Check 5: pcs_case must be greater than 0. A blank pcs_case or max_case_day is also an error (a blank mad is allowed).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1053" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B36" s="1053" t="inlineStr">
         <is>
-          <t>Change an Active part to Candidate</t>
+          <t>Change the status of a Candidate part</t>
         </is>
       </c>
       <c r="C36" s="1053" t="inlineStr">
         <is>
-          <t>PART-C</t>
+          <t>PART-I</t>
         </is>
       </c>
       <c r="D36" s="1054" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="E36" s="1054" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F36" s="1054" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G36" s="1053" t="inlineStr">
         <is>
-          <t>Candidate</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H36" s="1053" t="inlineStr">
@@ -50109,106 +50114,114 @@
           <t>E</t>
         </is>
       </c>
-      <c r="I36" s="1053" t="n"/>
+      <c r="I36" s="1053" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
       <c r="J36" s="1053" t="inlineStr">
         <is>
-          <t>Check 6: no part can be changed to Candidate.</t>
+          <t>Check 6: the status of a Candidate part cannot be changed by upload. Change it in the Edit part data modal.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1053" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B37" s="1053" t="inlineStr">
         <is>
-          <t>Add with a status</t>
+          <t>Change an Active part to Candidate</t>
         </is>
       </c>
       <c r="C37" s="1053" t="inlineStr">
         <is>
-          <t>PART-M03</t>
+          <t>PART-C</t>
         </is>
       </c>
       <c r="D37" s="1054" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="E37" s="1054" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F37" s="1054" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G37" s="1053" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="H37" s="1053" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I37" s="1053" t="inlineStr">
-        <is>
-          <t>14-Sep-2026</t>
-        </is>
-      </c>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="I37" s="1053" t="n"/>
       <c r="J37" s="1053" t="inlineStr">
         <is>
-          <t>Check 6: status of a new part is always Candidate, leave it blank.</t>
+          <t>Check 6: no part can be changed to Candidate.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1053" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B38" s="1053" t="inlineStr">
         <is>
-          <t>Add without effective date</t>
+          <t>Add with a status</t>
         </is>
       </c>
       <c r="C38" s="1053" t="inlineStr">
         <is>
-          <t>PART-M02</t>
+          <t>PART-M03</t>
         </is>
       </c>
       <c r="D38" s="1054" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="E38" s="1054" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F38" s="1054" t="n">
-        <v>40</v>
-      </c>
-      <c r="G38" s="1053" t="n"/>
+        <v>15</v>
+      </c>
+      <c r="G38" s="1053" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="H38" s="1053" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I38" s="1053" t="n"/>
+      <c r="I38" s="1053" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
       <c r="J38" s="1053" t="inlineStr">
         <is>
-          <t>Check 7: Effective Start Date is required for Candidate.</t>
+          <t>Check 6: status of a new part is always Candidate, leave it blank.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1053" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B39" s="1053" t="inlineStr">
         <is>
-          <t>Effective date in the past</t>
+          <t>Add without effective date</t>
         </is>
       </c>
       <c r="C39" s="1053" t="inlineStr">
@@ -50231,83 +50244,79 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I39" s="1053" t="inlineStr">
-        <is>
-          <t>12-Sep-2026</t>
-        </is>
-      </c>
+      <c r="I39" s="1053" t="n"/>
       <c r="J39" s="1053" t="inlineStr">
         <is>
-          <t>Check 7: Effective Start Date must be today or later.</t>
+          <t>Check 7: Effective Start Date is required for Candidate.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1053" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B40" s="1053" t="inlineStr">
         <is>
-          <t>Change effective date of an Active part</t>
+          <t>Effective date in the past</t>
         </is>
       </c>
       <c r="C40" s="1053" t="inlineStr">
         <is>
-          <t>PART-C</t>
+          <t>PART-M02</t>
         </is>
       </c>
       <c r="D40" s="1054" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="E40" s="1054" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F40" s="1054" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G40" s="1053" t="n"/>
       <c r="H40" s="1053" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I40" s="1053" t="inlineStr">
         <is>
-          <t>20-Sep-2026</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="J40" s="1053" t="inlineStr">
         <is>
-          <t>Check 8: effective date can only change while the part is Candidate.</t>
+          <t>Check 7: Effective Start Date must be today or later.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1053" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="B41" s="1053" t="inlineStr">
         <is>
-          <t>Max Case/Day below existing mapping</t>
+          <t>Change effective date of an Active part</t>
         </is>
       </c>
       <c r="C41" s="1053" t="inlineStr">
         <is>
-          <t>PART-A</t>
+          <t>PART-C</t>
         </is>
       </c>
       <c r="D41" s="1054" t="n">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="E41" s="1054" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="F41" s="1054" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G41" s="1053" t="n"/>
       <c r="H41" s="1053" t="inlineStr">
@@ -50315,52 +50324,52 @@
           <t>E</t>
         </is>
       </c>
-      <c r="I41" s="1053" t="n"/>
+      <c r="I41" s="1053" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="J41" s="1053" t="inlineStr">
         <is>
-          <t>Check 9: Max Case/Day 20 is below mapped 24. Reduce the mapping first in Mapping per Destination.</t>
+          <t>Check 8: effective date can only change while the part is Candidate.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1053" t="inlineStr">
         <is>
-          <t>E14</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B42" s="1053" t="inlineStr">
         <is>
-          <t>Valid row (= N1) mixed with an error row (= E2), row 1</t>
+          <t>Max Case/Day below existing mapping</t>
         </is>
       </c>
       <c r="C42" s="1053" t="inlineStr">
         <is>
-          <t>PART-M01</t>
+          <t>PART-A</t>
         </is>
       </c>
       <c r="D42" s="1054" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="E42" s="1054" t="n">
+        <v>60</v>
+      </c>
+      <c r="F42" s="1054" t="n">
         <v>20</v>
-      </c>
-      <c r="F42" s="1054" t="n">
-        <v>15</v>
       </c>
       <c r="G42" s="1053" t="n"/>
       <c r="H42" s="1053" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I42" s="1053" t="inlineStr">
-        <is>
-          <t>14-Sep-2026</t>
-        </is>
-      </c>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="I42" s="1053" t="n"/>
       <c r="J42" s="1053" t="inlineStr">
         <is>
-          <t>Whole file rejected. The valid row is NOT saved.</t>
+          <t>Check 9: Max Case/Day 20 is below mapped 24. Reduce the mapping first in Mapping per Destination.</t>
         </is>
       </c>
     </row>
@@ -50372,140 +50381,182 @@
       </c>
       <c r="B43" s="1053" t="inlineStr">
         <is>
-          <t>Valid row mixed with an error row, row 2</t>
+          <t>Valid row (= N1) mixed with an error row (= E2), row 1</t>
         </is>
       </c>
       <c r="C43" s="1053" t="inlineStr">
         <is>
-          <t>PART-Z99</t>
+          <t>PART-M01</t>
         </is>
       </c>
       <c r="D43" s="1054" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E43" s="1054" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F43" s="1054" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G43" s="1053" t="n"/>
       <c r="H43" s="1053" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I43" s="1053" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="J43" s="1053" t="inlineStr">
+        <is>
+          <t>Whole file rejected. The valid row is NOT saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1053" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="B44" s="1053" t="inlineStr">
+        <is>
+          <t>Valid row mixed with an error row, row 2</t>
+        </is>
+      </c>
+      <c r="C44" s="1053" t="inlineStr">
+        <is>
+          <t>PART-Z99</t>
+        </is>
+      </c>
+      <c r="D44" s="1054" t="n">
+        <v>100</v>
+      </c>
+      <c r="E44" s="1054" t="n">
+        <v>10</v>
+      </c>
+      <c r="F44" s="1054" t="n">
+        <v>10</v>
+      </c>
+      <c r="G44" s="1053" t="n"/>
+      <c r="H44" s="1053" t="inlineStr">
+        <is>
           <t>E</t>
         </is>
       </c>
-      <c r="I43" s="1053" t="n"/>
-      <c r="J43" s="1053" t="inlineStr">
+      <c r="I44" s="1053" t="n"/>
+      <c r="J44" s="1053" t="inlineStr">
         <is>
           <t>Check 2 on this row. Result report sheet Re-upload lists the rows to correct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1051" t="inlineStr">
-        <is>
-          <t>D. File-level errors (file check 4.1)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1052" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B46" s="1052" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="C46" s="1052" t="inlineStr">
-        <is>
-          <t>Expected result</t>
+      <c r="A46" s="1051" t="inlineStr">
+        <is>
+          <t>D. File-level errors (file check 4.1)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1053" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="B47" s="1053" t="inlineStr">
-        <is>
-          <t>File is .xls or .csv</t>
-        </is>
-      </c>
-      <c r="C47" s="1053" t="inlineStr">
-        <is>
-          <t>Rejected: file must be .xlsx.</t>
+      <c r="A47" s="1052" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B47" s="1052" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C47" s="1052" t="inlineStr">
+        <is>
+          <t>Expected result</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1053" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B48" s="1053" t="inlineStr">
         <is>
-          <t>File larger than 5 MB</t>
+          <t>File is .xls or .csv</t>
         </is>
       </c>
       <c r="C48" s="1053" t="inlineStr">
         <is>
-          <t>Rejected: file size exceeds 5 MB.</t>
+          <t>Rejected: file must be .xlsx.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1053" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B49" s="1053" t="inlineStr">
         <is>
-          <t>More than 5,000 data rows, or no data row</t>
+          <t>File larger than 5 MB</t>
         </is>
       </c>
       <c r="C49" s="1053" t="inlineStr">
         <is>
-          <t>Rejected: row count out of range.</t>
+          <t>Rejected: file size exceeds 5 MB.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1053" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B50" s="1053" t="inlineStr">
         <is>
-          <t>No sheet named Upload (e.g. only sheet Part List)</t>
+          <t>More than 5,000 data rows, or no data row</t>
         </is>
       </c>
       <c r="C50" s="1053" t="inlineStr">
         <is>
-          <t>Rejected: sheet Upload not found.</t>
+          <t>Rejected: row count out of range.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1053" t="inlineStr">
         <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B51" s="1053" t="inlineStr">
+        <is>
+          <t>No sheet named Upload (e.g. only sheet Part List)</t>
+        </is>
+      </c>
+      <c r="C51" s="1053" t="inlineStr">
+        <is>
+          <t>Rejected: sheet Upload not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1053" t="inlineStr">
+        <is>
           <t>F5</t>
         </is>
       </c>
-      <c r="B51" s="1053" t="inlineStr">
+      <c r="B52" s="1053" t="inlineStr">
         <is>
           <t>A template column is missing (e.g. flag_add_edit deleted)</t>
         </is>
       </c>
-      <c r="C51" s="1053" t="inlineStr">
+      <c r="C52" s="1053" t="inlineStr">
         <is>
           <t>Rejected: required column not found.</t>
         </is>

</xml_diff>